<commit_message>
Fit QFlex-T+ in the main pipeline where the paper uses it, inverse Gaussian N = 200 only, review fixes
</commit_message>
<xml_diff>
--- a/excel/InverseGaussian_vs_JohnsonSL_MC.xlsx
+++ b/excel/InverseGaussian_vs_JohnsonSL_MC.xlsx
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="16.5" customWidth="1" min="1" max="1"/>
@@ -763,7 +763,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1000 replicates per N. </t>
+          <t>N = 200, 1000 replicates (the paper runs the inverse Gaussian at N = 200 only).</t>
         </is>
       </c>
     </row>
@@ -1678,871 +1678,44 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>N = 50</t>
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="C35" s="13" t="inlineStr">
-        <is>
-          <t>Inverse Gaussian (μ = 0.919, λ = 1.069)</t>
-        </is>
-      </c>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="20" t="n"/>
-      <c r="G35" s="13" t="inlineStr">
-        <is>
-          <t>Johnson SL (ξ = 0, λ = 1, γ = 0.5, δ = 1.2)</t>
-        </is>
-      </c>
-      <c r="H35" s="19" t="n"/>
-      <c r="I35" s="20" t="n"/>
-      <c r="M35" s="13" t="inlineStr">
-        <is>
-          <t>Difference (IG - Johnson SL)</t>
-        </is>
-      </c>
-      <c r="N35" s="19" t="n"/>
-      <c r="O35" s="20" t="n"/>
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Design identical for both distributions: N = 200, 1000 replicates, K = 4, 7, 10, 13 shown (fitted 3-13); Log transform with the true lower bound 0.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="44" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Validity (%)</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>False Multimodality (%)</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Median W1 (%)</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Validity (%)</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>False Multimodality (%)</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>Median W1 (%)</t>
-        </is>
-      </c>
-      <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Validity (%)</t>
-        </is>
-      </c>
-      <c r="N36" s="3" t="inlineStr">
-        <is>
-          <t>False Multimodality (%)</t>
-        </is>
-      </c>
-      <c r="O36" s="3" t="inlineStr">
-        <is>
-          <t>Median W1 (%)</t>
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>Replicate r of the inverse Gaussian uses the same uniforms as Johnson SL replicate r (seed 42 + N*1000 + r), pushed through the IG quantile function.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Metalog</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C37" s="6" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="D37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>3.39</v>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="H37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="7" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="M37" s="17">
-        <f>C37-G37</f>
-        <v/>
-      </c>
-      <c r="N37" s="17">
-        <f>D37-H37</f>
-        <v/>
-      </c>
-      <c r="O37" s="18">
-        <f>E37-I37</f>
-        <v/>
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Inverse Gaussian parameters (mu = 0.919, lambda = 1.069). Johnson SL = the Section 4.1 reference distribution.</t>
+        </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="E38" s="7" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="G38" s="6" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="H38" s="6" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="I38" s="7" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="M38" s="17">
-        <f>C38-G38</f>
-        <v/>
-      </c>
-      <c r="N38" s="17">
-        <f>D38-H38</f>
-        <v/>
-      </c>
-      <c r="O38" s="18">
-        <f>E38-I38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>33.2</v>
-      </c>
-      <c r="D39" s="6" t="n">
-        <v>90.09999999999999</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="G39" s="6" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>91.90000000000001</v>
-      </c>
-      <c r="I39" s="7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="M39" s="17">
-        <f>C39-G39</f>
-        <v/>
-      </c>
-      <c r="N39" s="17">
-        <f>D39-H39</f>
-        <v/>
-      </c>
-      <c r="O39" s="18">
-        <f>E39-I39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="D40" s="6" t="n">
-        <v>99</v>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="G40" s="6" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="H40" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="I40" s="7" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="M40" s="17">
-        <f>C40-G40</f>
-        <v/>
-      </c>
-      <c r="N40" s="17">
-        <f>D40-H40</f>
-        <v/>
-      </c>
-      <c r="O40" s="18">
-        <f>E40-I40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>QFlex-U</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>98.09999999999999</v>
-      </c>
-      <c r="D41" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="G41" s="6" t="n">
-        <v>99.2</v>
-      </c>
-      <c r="H41" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="7" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="M41" s="17">
-        <f>C41-G41</f>
-        <v/>
-      </c>
-      <c r="N41" s="17">
-        <f>D41-H41</f>
-        <v/>
-      </c>
-      <c r="O41" s="18">
-        <f>E41-I41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C42" s="6" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="D42" s="6" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="E42" s="7" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="G42" s="6" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="I42" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="M42" s="17">
-        <f>C42-G42</f>
-        <v/>
-      </c>
-      <c r="N42" s="17">
-        <f>D42-H42</f>
-        <v/>
-      </c>
-      <c r="O42" s="18">
-        <f>E42-I42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n"/>
-      <c r="B43" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="D43" s="6" t="n">
-        <v>92.2</v>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="G43" s="6" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="H43" s="6" t="n">
-        <v>90.7</v>
-      </c>
-      <c r="I43" s="7" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="M43" s="17">
-        <f>C43-G43</f>
-        <v/>
-      </c>
-      <c r="N43" s="17">
-        <f>D43-H43</f>
-        <v/>
-      </c>
-      <c r="O43" s="18">
-        <f>E43-I43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C44" s="6" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="D44" s="6" t="n">
-        <v>97.7</v>
-      </c>
-      <c r="E44" s="7" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G44" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H44" s="6" t="n">
-        <v>98</v>
-      </c>
-      <c r="I44" s="7" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="M44" s="17">
-        <f>C44-G44</f>
-        <v/>
-      </c>
-      <c r="N44" s="17">
-        <f>D44-H44</f>
-        <v/>
-      </c>
-      <c r="O44" s="18">
-        <f>E44-I44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>QFlex-T+</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D45" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" s="7" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="G45" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H45" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" s="7" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="M45" s="17">
-        <f>C45-G45</f>
-        <v/>
-      </c>
-      <c r="N45" s="17">
-        <f>D45-H45</f>
-        <v/>
-      </c>
-      <c r="O45" s="18">
-        <f>E45-I45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n"/>
-      <c r="B46" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C46" s="6" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="D46" s="6" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="E46" s="7" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="G46" s="6" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="H46" s="6" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="M46" s="17">
-        <f>C46-G46</f>
-        <v/>
-      </c>
-      <c r="N46" s="17">
-        <f>D46-H46</f>
-        <v/>
-      </c>
-      <c r="O46" s="18">
-        <f>E46-I46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C47" s="6" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="D47" s="6" t="n">
-        <v>83.7</v>
-      </c>
-      <c r="E47" s="7" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="G47" s="6" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="H47" s="6" t="n">
-        <v>87.40000000000001</v>
-      </c>
-      <c r="I47" s="7" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="M47" s="17">
-        <f>C47-G47</f>
-        <v/>
-      </c>
-      <c r="N47" s="17">
-        <f>D47-H47</f>
-        <v/>
-      </c>
-      <c r="O47" s="18">
-        <f>E47-I47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n"/>
-      <c r="B48" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="D48" s="6" t="n">
-        <v>98.8</v>
-      </c>
-      <c r="E48" s="7" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="G48" s="6" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="H48" s="6" t="n">
-        <v>97.90000000000001</v>
-      </c>
-      <c r="I48" s="7" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="M48" s="17">
-        <f>C48-G48</f>
-        <v/>
-      </c>
-      <c r="N48" s="17">
-        <f>D48-H48</f>
-        <v/>
-      </c>
-      <c r="O48" s="18">
-        <f>E48-I48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>QFlex-TA+</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C49" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D49" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="7" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="G49" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H49" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" s="7" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="M49" s="17">
-        <f>C49-G49</f>
-        <v/>
-      </c>
-      <c r="N49" s="17">
-        <f>D49-H49</f>
-        <v/>
-      </c>
-      <c r="O49" s="18">
-        <f>E49-I49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D50" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E50" s="7" t="n">
-        <v>2.86</v>
-      </c>
-      <c r="G50" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H50" s="6" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="I50" s="7" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="M50" s="17">
-        <f>C50-G50</f>
-        <v/>
-      </c>
-      <c r="N50" s="17">
-        <f>D50-H50</f>
-        <v/>
-      </c>
-      <c r="O50" s="18">
-        <f>E50-I50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C51" s="6" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="D51" s="6" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="E51" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G51" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H51" s="6" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="I51" s="7" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="M51" s="17">
-        <f>C51-G51</f>
-        <v/>
-      </c>
-      <c r="N51" s="17">
-        <f>D51-H51</f>
-        <v/>
-      </c>
-      <c r="O51" s="18">
-        <f>E51-I51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n"/>
-      <c r="B52" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C52" s="6" t="n">
-        <v>97.59999999999999</v>
-      </c>
-      <c r="D52" s="6" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="G52" s="6" t="n">
-        <v>97.5</v>
-      </c>
-      <c r="H52" s="6" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="I52" s="7" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="M52" s="17">
-        <f>C52-G52</f>
-        <v/>
-      </c>
-      <c r="N52" s="17">
-        <f>D52-H52</f>
-        <v/>
-      </c>
-      <c r="O52" s="18">
-        <f>E52-I52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>QFlex-A+</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C53" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="7" t="n">
-        <v>3.44</v>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="7" t="n">
-        <v>3.62</v>
-      </c>
-      <c r="M53" s="17">
-        <f>C53-G53</f>
-        <v/>
-      </c>
-      <c r="N53" s="17">
-        <f>D53-H53</f>
-        <v/>
-      </c>
-      <c r="O53" s="18">
-        <f>E53-I53</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C54" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D54" s="6" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="E54" s="7" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="I54" s="7" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="M54" s="17">
-        <f>C54-G54</f>
-        <v/>
-      </c>
-      <c r="N54" s="17">
-        <f>D54-H54</f>
-        <v/>
-      </c>
-      <c r="O54" s="18">
-        <f>E54-I54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C55" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D55" s="6" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E55" s="7" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="I55" s="7" t="n">
-        <v>2.86</v>
-      </c>
-      <c r="M55" s="17">
-        <f>C55-G55</f>
-        <v/>
-      </c>
-      <c r="N55" s="17">
-        <f>D55-H55</f>
-        <v/>
-      </c>
-      <c r="O55" s="18">
-        <f>E55-I55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="n"/>
-      <c r="B56" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C56" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D56" s="6" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="E56" s="7" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="G56" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="I56" s="7" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="M56" s="17">
-        <f>C56-G56</f>
-        <v/>
-      </c>
-      <c r="N56" s="17">
-        <f>D56-H56</f>
-        <v/>
-      </c>
-      <c r="O56" s="18">
-        <f>E56-I56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="11" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
-        <is>
-          <t>Design identical for both distributions: N = 50 and 200, 1000 replicates, K = 4, 7, 10, 13 shown (fitted 3-13); Log transform with the true lower bound 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
-        <is>
-          <t>Replicate r of the inverse Gaussian uses the same uniforms as Johnson SL replicate r (seed 42 + N*1000 + r), pushed through the IG quantile function.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr">
-        <is>
-          <t>Inverse Gaussian parameters (mu = 0.919, lambda = 1.069). Johnson SL = the Section 4.1 reference distribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="12" t="n"/>
-    </row>
+      <c r="A38" s="12" t="n"/>
+    </row>
+    <row r="39"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="3">
     <mergeCell ref="G10:I10"/>
     <mergeCell ref="M10:O10"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="C35:E35"/>
     <mergeCell ref="C10:E10"/>
   </mergeCells>
   <conditionalFormatting sqref="M12:O31">

</xml_diff>